<commit_message>
Docs: README completo com fotos do Dashboard e Exel
</commit_message>
<xml_diff>
--- a/relatorio_vendas.xlsx
+++ b/relatorio_vendas.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -804,6 +804,62 @@
         <v>8765.120000000001</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>37</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>46090.58914172406</v>
+      </c>
+      <c r="D27" t="n">
+        <v>980.8099999999999</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>42</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>46090.60232124857</v>
+      </c>
+      <c r="D28" t="n">
+        <v>5665.44</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>46090.60476155933</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3613.29</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>46090.60732524037</v>
+      </c>
+      <c r="D30" t="n">
+        <v>944.24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>